<commit_message>
Daily EOD data and reports for 2026-10-28
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20261028.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20261028.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.615</v>
+        <v>1.625</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.065</v>
+        <v>0.075</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.19%</t>
+          <t>4.84%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>247387.32</v>
+        <v>248919.12</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>9956.76</v>
+        <v>11488.57</v>
       </c>
     </row>
     <row r="5">
@@ -542,24 +542,24 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>58.305</v>
+        <v>58.38</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.315</v>
+        <v>0.39</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.54%</t>
+          <t>0.67%</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
         <v>8000</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>466440</v>
+        <v>467040</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>2520</v>
+        <v>3120</v>
       </c>
     </row>
     <row r="7">
@@ -596,14 +596,14 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>163.71</v>
+        <v>164.22</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>1.69</v>
+        <v>2.2</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.04%</t>
+          <t>1.36%</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>198.3</v>
+        <v>198.26</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>1.52</v>
+        <v>1.48</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.77%</t>
+          <t>0.75%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>793200</v>
+        <v>793040</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>6080</v>
+        <v>5920</v>
       </c>
     </row>
     <row r="11">
@@ -704,24 +704,24 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>11.72</v>
+        <v>11.98</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>1.1</v>
+        <v>1.36</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>10.36%</t>
+          <t>12.81%</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
         <v>3045</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>35687.4</v>
+        <v>36479.1</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>3349.5</v>
+        <v>4141.2</v>
       </c>
     </row>
     <row r="13">
@@ -758,24 +758,24 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0</v>
+        <v>0.078</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>-0.08</v>
+        <v>-0.002</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>-2.50%</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
         <v>9412</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>0</v>
+        <v>734.14</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>-752.96</v>
+        <v>-18.82</v>
       </c>
     </row>
     <row r="15">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>36.34</v>
+        <v>36.59</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.16</v>
+        <v>0.41</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0.44%</t>
+          <t>1.13%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>32.68</v>
+        <v>32.395</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>-0.5</v>
+        <v>-0.785</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>-1.51%</t>
+          <t>-2.37%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>42091.84</v>
+        <v>41724.76</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>-644</v>
+        <v>-1011.08</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1764856.55</v>
+        <v>1767987.12</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>14984.86</v>
+        <v>18115.42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>